<commit_message>
columnType: the riInstallationMethod conditions test the enumeration's spaced values (full displacement, partial displacement)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/columnType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/columnType.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -995,7 +995,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement']</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement' or .='partial_displacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement' or .='partial displacement']</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement' or .='partial_displacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement' or .='partial displacement']</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement' or .='replacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement' or .='replacement']</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement' or .='replacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement' or .='replacement']</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full_displacement' or .='replacement']</t>
+          <t>ancestor::diggs:RIColumn/diggs:riInstallationMethod[.='full displacement' or .='replacement']</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full_displacement' or .='replacement']</t>
+          <t>ancestor::diggs:RIColumnSpecification/diggs:riInstallationMethod[.='full displacement' or .='replacement']</t>
         </is>
       </c>
     </row>

</xml_diff>